<commit_message>
#1 Parts placement in-progress.
</commit_message>
<xml_diff>
--- a/Design_Files/BOM/Client_BOM.xlsx
+++ b/Design_Files/BOM/Client_BOM.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\manarharake-palmpcb\Design_Files\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LiberDB\Documents\GitHub\manarharake-palmpcb\Design_Files\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -72,9 +72,6 @@
     <t>C2</t>
   </si>
   <si>
-    <t>C4, C5, C6, C7, C8, C9, C12, C15, C19, C21, C24, C25, C27</t>
-  </si>
-  <si>
     <t>C10</t>
   </si>
   <si>
@@ -114,9 +111,6 @@
     <t>J5, J6, J7, J8, J9, J10</t>
   </si>
   <si>
-    <t>J11</t>
-  </si>
-  <si>
     <t>LED1, LED2</t>
   </si>
   <si>
@@ -222,9 +216,6 @@
     <t>Slide Lock 5P Bottom Contact Surface Mount，Right Angle 1mm SMD,P=1mm,Surface Mount，Right Angle FFC/FPC Connectors ROHS</t>
   </si>
   <si>
-    <t>CONN RCP USB3.1 TYPEC 24P SMD RA</t>
-  </si>
-  <si>
     <t>blue 0603 Light Emitting Diodes (LED) ROHS</t>
   </si>
   <si>
@@ -366,9 +357,6 @@
     <t>ESD5302F-3/TR</t>
   </si>
   <si>
-    <t>2305018-2</t>
-  </si>
-  <si>
     <t>NCD0603B3</t>
   </si>
   <si>
@@ -450,9 +438,6 @@
     <t>JUSHUO</t>
   </si>
   <si>
-    <t>TE Connectivity AMP</t>
-  </si>
-  <si>
     <t>Foshan NationStar Optoelectronics</t>
   </si>
   <si>
@@ -541,6 +526,21 @@
   </si>
   <si>
     <t>Custom</t>
+  </si>
+  <si>
+    <t>J4</t>
+  </si>
+  <si>
+    <t>5A 1 16P Female Type-C SMD USB Connectors ROHS</t>
+  </si>
+  <si>
+    <t>TYPE-C-31-M-12</t>
+  </si>
+  <si>
+    <t>Korean Hroparts Elec</t>
+  </si>
+  <si>
+    <t>C4, C5, C6, C7, C8, C9, C12, C15, C19, C24, C25, C27</t>
   </si>
 </sst>
 </file>
@@ -1073,25 +1073,25 @@
         <v>14</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1107,19 +1107,19 @@
         <v>15</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="J3" s="7">
         <v>2</v>
@@ -1139,19 +1139,19 @@
         <v>16</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="J4" s="9">
         <v>1</v>
@@ -1168,25 +1168,25 @@
         <v>2</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>17</v>
+        <v>173</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="J5" s="7">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K5" s="7"/>
     </row>
@@ -1200,22 +1200,22 @@
         <v>2</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="J6" s="9">
         <v>1</v>
@@ -1232,22 +1232,22 @@
         <v>2</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="J7" s="7">
         <v>3</v>
@@ -1264,22 +1264,22 @@
         <v>2</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="J8" s="9">
         <v>3</v>
@@ -1296,22 +1296,22 @@
         <v>2</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
@@ -1328,22 +1328,22 @@
         <v>2</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="J10" s="9">
         <v>4</v>
@@ -1360,22 +1360,22 @@
         <v>2</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="J11" s="7">
         <v>2</v>
@@ -1392,22 +1392,22 @@
         <v>3</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
@@ -1424,22 +1424,22 @@
         <v>3</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="J13" s="7">
         <v>2</v>
@@ -1456,22 +1456,22 @@
         <v>3</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
@@ -1488,22 +1488,22 @@
         <v>4</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
@@ -1520,22 +1520,22 @@
         <v>5</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="G16" s="10">
         <v>1729128</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="J16" s="9">
         <v>1</v>
@@ -1549,25 +1549,25 @@
         <v>15</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="I17" s="10" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="J17" s="7">
         <v>1</v>
@@ -1584,29 +1584,29 @@
         <v>6</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="J18" s="9">
         <v>6</v>
       </c>
       <c r="K18" s="9"/>
     </row>
-    <row r="19" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="11">
         <f>ROW(B19) - ROW($B$2)</f>
@@ -1615,23 +1615,23 @@
       <c r="C19" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="D19" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="E19" s="8" t="s">
-        <v>67</v>
+      <c r="D19" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>170</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>173</v>
-      </c>
-      <c r="G19" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="H19" s="7" t="s">
-        <v>143</v>
+        <v>168</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="H19" s="9" t="s">
+        <v>172</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="J19" s="7">
         <v>1</v>
@@ -1648,22 +1648,22 @@
         <v>8</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="J20" s="9">
         <v>2</v>
@@ -1680,22 +1680,22 @@
         <v>8</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="J21" s="7">
         <v>2</v>
@@ -1712,22 +1712,22 @@
         <v>9</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="J22" s="9">
         <v>7</v>
@@ -1744,22 +1744,22 @@
         <v>9</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="J23" s="7">
         <v>1</v>
@@ -1776,22 +1776,22 @@
         <v>9</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="J24" s="9">
         <v>4</v>
@@ -1808,22 +1808,22 @@
         <v>9</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="J25" s="7">
         <v>2</v>
@@ -1840,22 +1840,22 @@
         <v>9</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="J26" s="9">
         <v>2</v>
@@ -1872,22 +1872,22 @@
         <v>10</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="J27" s="7">
         <v>2</v>
@@ -1904,22 +1904,22 @@
         <v>9</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="J28" s="9">
         <v>1</v>
@@ -1936,22 +1936,22 @@
         <v>9</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
@@ -1968,22 +1968,22 @@
         <v>9</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="J30" s="9">
         <v>2</v>
@@ -2000,22 +2000,22 @@
         <v>9</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="J31" s="7">
         <v>1</v>
@@ -2032,22 +2032,22 @@
         <v>9</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="J32" s="9">
         <v>1</v>
@@ -2064,22 +2064,22 @@
         <v>11</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
@@ -2096,22 +2096,22 @@
         <v>12</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="I34" s="8" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="J34" s="9">
         <v>1</v>
@@ -2128,22 +2128,22 @@
         <v>12</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="J35" s="7">
         <v>3</v>
@@ -2160,22 +2160,22 @@
         <v>12</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="I36" s="8" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="J36" s="9">
         <v>1</v>
@@ -2192,22 +2192,22 @@
         <v>13</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="G37" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="H37" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="H37" s="7" t="s">
-        <v>136</v>
-      </c>
       <c r="I37" s="8" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="J37" s="7">
         <v>1</v>

</xml_diff>

<commit_message>
#1 BOM's updated with FPC Part No. : Re-routing in-progress.
</commit_message>
<xml_diff>
--- a/Design_Files/BOM/Client_BOM.xlsx
+++ b/Design_Files/BOM/Client_BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MarsVirgo\Documents\GitHub\manarharake-palmpcb\Design_Files\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCB7F524-ED55-459C-899F-55FA0C58FEE5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C78B4A20-C49E-46B3-B725-CBA727560F5D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7545" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -124,9 +124,6 @@
     <t>R12, R14</t>
   </si>
   <si>
-    <t>R17</t>
-  </si>
-  <si>
     <t>R20</t>
   </si>
   <si>
@@ -196,9 +193,6 @@
     <t>2mm pitch Solder Pad</t>
   </si>
   <si>
-    <t>Slide Lock 5P Bottom Contact Surface Mount，Right Angle 1mm SMD,P=1mm,Surface Mount，Right Angle FFC/FPC Connectors ROHS</t>
-  </si>
-  <si>
     <t>blue 0603 Light Emitting Diodes (LED) ROHS</t>
   </si>
   <si>
@@ -274,9 +268,6 @@
     <t>PH-01291</t>
   </si>
   <si>
-    <t>AFA07-S05FCC-00</t>
-  </si>
-  <si>
     <t>LED-0603</t>
   </si>
   <si>
@@ -415,9 +406,6 @@
     <t>Liansheng</t>
   </si>
   <si>
-    <t>JUSHUO</t>
-  </si>
-  <si>
     <t>Foshan NationStar Optoelectronics</t>
   </si>
   <si>
@@ -527,6 +515,18 @@
   </si>
   <si>
     <t>U6</t>
+  </si>
+  <si>
+    <t>Ra</t>
+  </si>
+  <si>
+    <t>1.0-5PXJPZ</t>
+  </si>
+  <si>
+    <t>BOOMELE(Boom Precision Elec)</t>
+  </si>
+  <si>
+    <t>Slide Lock -25℃~+85℃ 5P Bottom Contact Surface Mount，Right Angle 1mm SMD,P=1mm,Surface Mount，Right Angle FFC/FPC Connectors ROHS</t>
   </si>
 </sst>
 </file>
@@ -1059,25 +1059,25 @@
         <v>12</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="J2" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="K2" s="5" t="s">
         <v>156</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1093,19 +1093,19 @@
         <v>13</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="J3" s="7">
         <v>2</v>
@@ -1125,19 +1125,19 @@
         <v>14</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="J4" s="9">
         <v>1</v>
@@ -1154,22 +1154,22 @@
         <v>2</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="J5" s="7">
         <v>12</v>
@@ -1189,19 +1189,19 @@
         <v>15</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="J6" s="9">
         <v>1</v>
@@ -1221,19 +1221,19 @@
         <v>16</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="J7" s="7">
         <v>3</v>
@@ -1253,19 +1253,19 @@
         <v>17</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="J8" s="9">
         <v>3</v>
@@ -1285,19 +1285,19 @@
         <v>18</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
@@ -1314,22 +1314,22 @@
         <v>2</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="J10" s="9">
         <v>2</v>
@@ -1349,19 +1349,19 @@
         <v>19</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="J11" s="7">
         <v>2</v>
@@ -1381,19 +1381,19 @@
         <v>20</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
@@ -1413,19 +1413,19 @@
         <v>21</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="J13" s="7">
         <v>2</v>
@@ -1445,19 +1445,19 @@
         <v>22</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
@@ -1477,19 +1477,19 @@
         <v>23</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
@@ -1503,32 +1503,32 @@
         <v>14</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>24</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="J16" s="7">
         <v>1</v>
       </c>
       <c r="K16" s="7"/>
     </row>
-    <row r="17" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="11">
         <f t="shared" si="0"/>
@@ -1540,20 +1540,20 @@
       <c r="D17" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E17" s="10" t="s">
-        <v>58</v>
+      <c r="E17" s="8" t="s">
+        <v>168</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="H17" s="9" t="s">
-        <v>131</v>
+        <v>166</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>167</v>
       </c>
       <c r="I17" s="10" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="J17" s="9">
         <v>6</v>
@@ -1570,22 +1570,22 @@
         <v>6</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="F18" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="G18" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="H18" s="9" t="s">
         <v>161</v>
       </c>
-      <c r="G18" s="10" t="s">
-        <v>164</v>
-      </c>
-      <c r="H18" s="9" t="s">
-        <v>165</v>
-      </c>
       <c r="I18" s="10" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="J18" s="7">
         <v>1</v>
@@ -1605,19 +1605,19 @@
         <v>26</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="J19" s="9">
         <v>2</v>
@@ -1637,19 +1637,19 @@
         <v>27</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="J20" s="7">
         <v>2</v>
@@ -1669,19 +1669,19 @@
         <v>28</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="H21" s="9" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="J21" s="9">
         <v>7</v>
@@ -1701,19 +1701,19 @@
         <v>29</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I22" s="8" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="J22" s="7">
         <v>1</v>
@@ -1733,19 +1733,19 @@
         <v>30</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G23" s="10" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="H23" s="9" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I23" s="10" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="J23" s="9">
         <v>4</v>
@@ -1765,19 +1765,19 @@
         <v>31</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I24" s="8" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="J24" s="7">
         <v>2</v>
@@ -1797,19 +1797,19 @@
         <v>32</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G25" s="10" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="H25" s="9" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I25" s="10" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="J25" s="9">
         <v>2</v>
@@ -1829,19 +1829,19 @@
         <v>33</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I26" s="8" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="J26" s="7">
         <v>2</v>
@@ -1858,22 +1858,22 @@
         <v>8</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>34</v>
+        <v>165</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="G27" s="10" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="H27" s="9" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I27" s="10" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="J27" s="9">
         <v>1</v>
@@ -1890,22 +1890,22 @@
         <v>8</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G28" s="8" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="H28" s="7" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="J28" s="7">
         <v>1</v>
@@ -1922,22 +1922,22 @@
         <v>8</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F29" s="9" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G29" s="10" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="H29" s="9" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I29" s="10" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="J29" s="9">
         <v>2</v>
@@ -1954,22 +1954,22 @@
         <v>8</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G30" s="8" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="H30" s="7" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I30" s="8" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="J30" s="7">
         <v>1</v>
@@ -1986,22 +1986,22 @@
         <v>8</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G31" s="10" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H31" s="9" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="I31" s="10" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="J31" s="9">
         <v>1</v>
@@ -2018,22 +2018,22 @@
         <v>10</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="G32" s="8" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="H32" s="7" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="I32" s="8" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="J32" s="7">
         <v>1</v>
@@ -2050,22 +2050,22 @@
         <v>10</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="G33" s="10" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="H33" s="9" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="J33" s="9">
         <v>1</v>
@@ -2082,22 +2082,22 @@
         <v>10</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G34" s="8" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="H34" s="7" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="I34" s="8" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="J34" s="7">
         <v>3</v>
@@ -2114,22 +2114,22 @@
         <v>10</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="G35" s="10" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="H35" s="9" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="J35" s="9">
         <v>1</v>
@@ -2146,22 +2146,22 @@
         <v>11</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="G36" s="8" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="H36" s="7" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="I36" s="8" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="J36" s="7">
         <v>1</v>
@@ -2172,7 +2172,10 @@
   <mergeCells count="1">
     <mergeCell ref="I1:K1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="H17" r:id="rId1" display="https://www.lcsc.com/brand-detail/86.html" xr:uid="{2653AC96-EB3F-456C-A7DE-191DEDF3D541}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#1 @MarsVirgo Client and JLCPCB BOM Updated.
</commit_message>
<xml_diff>
--- a/Design_Files/BOM/Client_BOM.xlsx
+++ b/Design_Files/BOM/Client_BOM.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20410"/>
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MarsVirgo\Documents\GitHub\manarharake-palmpcb\Design_Files\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\manarharake-palmpcb\Design_Files\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C78B4A20-C49E-46B3-B725-CBA727560F5D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7545" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7545"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
@@ -532,7 +531,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1017,7 +1016,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:K36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1032,6 +1031,9 @@
     <col min="9" max="9" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1528,69 +1530,69 @@
       </c>
       <c r="K16" s="7"/>
     </row>
-    <row r="17" spans="1:11" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B17) - ROW($B$2)</f>
         <v>15</v>
       </c>
-      <c r="C17" s="13" t="s">
-        <v>5</v>
+      <c r="C17" s="12" t="s">
+        <v>6</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>168</v>
+        <v>158</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>159</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>157</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>166</v>
-      </c>
-      <c r="H17" s="7" t="s">
-        <v>167</v>
+        <v>160</v>
+      </c>
+      <c r="H17" s="9" t="s">
+        <v>161</v>
       </c>
       <c r="I17" s="10" t="s">
         <v>153</v>
       </c>
-      <c r="J17" s="9">
-        <v>6</v>
-      </c>
-      <c r="K17" s="9"/>
-    </row>
-    <row r="18" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J17" s="7">
+        <v>1</v>
+      </c>
+      <c r="K17" s="7"/>
+    </row>
+    <row r="18" spans="1:11" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="11">
-        <f>ROW(B18) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C18" s="12" t="s">
-        <v>6</v>
+      <c r="C18" s="13" t="s">
+        <v>5</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>158</v>
-      </c>
-      <c r="E18" s="10" t="s">
-        <v>159</v>
+        <v>25</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>168</v>
       </c>
       <c r="F18" s="7" t="s">
         <v>157</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>160</v>
-      </c>
-      <c r="H18" s="9" t="s">
-        <v>161</v>
+        <v>166</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>167</v>
       </c>
       <c r="I18" s="10" t="s">
         <v>153</v>
       </c>
-      <c r="J18" s="7">
-        <v>1</v>
-      </c>
-      <c r="K18" s="7"/>
+      <c r="J18" s="9">
+        <v>6</v>
+      </c>
+      <c r="K18" s="9"/>
     </row>
     <row r="19" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
@@ -1851,157 +1853,157 @@
     <row r="27" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B27) - ROW($B$2)</f>
         <v>25</v>
       </c>
-      <c r="C27" s="13" t="s">
+      <c r="C27" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="D27" s="9" t="s">
-        <v>165</v>
-      </c>
-      <c r="E27" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="F27" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="G27" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="H27" s="9" t="s">
+      <c r="D27" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="G27" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="H27" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="I27" s="10" t="s">
-        <v>147</v>
-      </c>
-      <c r="J27" s="9">
+      <c r="I27" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="J27" s="7">
         <v>1</v>
       </c>
-      <c r="K27" s="9"/>
+      <c r="K27" s="7"/>
     </row>
     <row r="28" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="11">
-        <f>ROW(B28) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C28" s="12" t="s">
+      <c r="C28" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D28" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="E28" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="F28" s="7" t="s">
+      <c r="D28" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E28" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="F28" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="G28" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="H28" s="7" t="s">
+      <c r="G28" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="H28" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="I28" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="J28" s="7">
-        <v>1</v>
-      </c>
-      <c r="K28" s="7"/>
+      <c r="I28" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="J28" s="9">
+        <v>2</v>
+      </c>
+      <c r="K28" s="9"/>
     </row>
     <row r="29" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B29) - ROW($B$2)</f>
         <v>27</v>
       </c>
-      <c r="C29" s="13" t="s">
+      <c r="C29" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="D29" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E29" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="F29" s="9" t="s">
+      <c r="D29" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="F29" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="G29" s="10" t="s">
-        <v>112</v>
-      </c>
-      <c r="H29" s="9" t="s">
+      <c r="G29" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="H29" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="I29" s="10" t="s">
-        <v>149</v>
-      </c>
-      <c r="J29" s="9">
-        <v>2</v>
-      </c>
-      <c r="K29" s="9"/>
-    </row>
-    <row r="30" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I29" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="J29" s="7">
+        <v>1</v>
+      </c>
+      <c r="K29" s="7"/>
+    </row>
+    <row r="30" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="11">
-        <f>ROW(B30) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="C30" s="12" t="s">
+      <c r="C30" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D30" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="E30" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="F30" s="7" t="s">
+      <c r="D30" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E30" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="F30" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="G30" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="H30" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="I30" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="J30" s="7">
+      <c r="G30" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="H30" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="I30" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="J30" s="9">
         <v>1</v>
       </c>
-      <c r="K30" s="7"/>
-    </row>
-    <row r="31" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K30" s="9"/>
+    </row>
+    <row r="31" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B31) - ROW($B$2)</f>
         <v>29</v>
       </c>
       <c r="C31" s="13" t="s">
         <v>8</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>37</v>
+        <v>165</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G31" s="10" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="H31" s="9" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="I31" s="10" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="J31" s="9">
         <v>1</v>
@@ -2173,7 +2175,7 @@
     <mergeCell ref="I1:K1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="H17" r:id="rId1" display="https://www.lcsc.com/brand-detail/86.html" xr:uid="{2653AC96-EB3F-456C-A7DE-191DEDF3D541}"/>
+    <hyperlink ref="H18" r:id="rId1" display="https://www.lcsc.com/brand-detail/86.html"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>

</xml_diff>

<commit_message>
#1 Connector update in Client and JLCPCB BOM.
</commit_message>
<xml_diff>
--- a/Design_Files/BOM/Client_BOM.xlsx
+++ b/Design_Files/BOM/Client_BOM.xlsx
@@ -519,13 +519,13 @@
     <t>Ra</t>
   </si>
   <si>
-    <t>1.0-5PXJPZ</t>
-  </si>
-  <si>
-    <t>BOOMELE(Boom Precision Elec)</t>
-  </si>
-  <si>
-    <t>Slide Lock -25℃~+85℃ 5P Bottom Contact Surface Mount，Right Angle 1mm SMD,P=1mm,Surface Mount，Right Angle FFC/FPC Connectors ROHS</t>
+    <t>CONN FFC FPC BOTTOM 5POS 1MM R/A</t>
+  </si>
+  <si>
+    <t>SFW5R-1STE1LF</t>
+  </si>
+  <si>
+    <t>Amphenol ICC / FCI</t>
   </si>
 </sst>
 </file>
@@ -1562,7 +1562,7 @@
       </c>
       <c r="K17" s="7"/>
     </row>
-    <row r="18" spans="1:11" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="11">
         <f t="shared" si="0"/>
@@ -1574,17 +1574,17 @@
       <c r="D18" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E18" s="8" t="s">
-        <v>168</v>
+      <c r="E18" s="10" t="s">
+        <v>166</v>
       </c>
       <c r="F18" s="7" t="s">
         <v>157</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>166</v>
-      </c>
-      <c r="H18" s="7" t="s">
         <v>167</v>
+      </c>
+      <c r="H18" s="9" t="s">
+        <v>168</v>
       </c>
       <c r="I18" s="10" t="s">
         <v>153</v>

</xml_diff>

<commit_message>
#1 PCB Completed: Fresh Deliverables generated.
</commit_message>
<xml_diff>
--- a/Design_Files/BOM/Client_BOM.xlsx
+++ b/Design_Files/BOM/Client_BOM.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\manarharake-palmpcb\Design_Files\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LiberDB\Documents\GitHub\manarharake-palmpcb\Design_Files\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -180,9 +180,6 @@
     <t>TVS DIODE 5VWM 6.3VC DSN0603-2</t>
   </si>
   <si>
-    <t>DIODE SCHOTTKY 60V 2A SMA</t>
-  </si>
-  <si>
     <t>16A 20V 7V 5V@Max Unidirectional SOT-23 TVS ROHS</t>
   </si>
   <si>
@@ -258,9 +255,6 @@
     <t>DSN0603-2</t>
   </si>
   <si>
-    <t>SMA</t>
-  </si>
-  <si>
     <t>Sot-23</t>
   </si>
   <si>
@@ -324,9 +318,6 @@
     <t>PESD5V0H1BSFYL</t>
   </si>
   <si>
-    <t>B260A-13-F</t>
-  </si>
-  <si>
     <t>ESD5302F-3/TR</t>
   </si>
   <si>
@@ -396,9 +387,6 @@
     <t>Nexperia</t>
   </si>
   <si>
-    <t>Diodes</t>
-  </si>
-  <si>
     <t>WILLSEMI</t>
   </si>
   <si>
@@ -526,6 +514,18 @@
   </si>
   <si>
     <t>Amphenol ICC / FCI</t>
+  </si>
+  <si>
+    <t>SS54B-HF</t>
+  </si>
+  <si>
+    <t>Comchip</t>
+  </si>
+  <si>
+    <t>SMB</t>
+  </si>
+  <si>
+    <t>40V 5A 550mV@5A DO-214AA(SMB) Schottky Barrier Diodes (SBD) ROHS</t>
   </si>
 </sst>
 </file>
@@ -1064,22 +1064,22 @@
         <v>42</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="J2" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="K2" s="5" t="s">
         <v>152</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1098,16 +1098,16 @@
         <v>43</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="J3" s="7">
         <v>2</v>
@@ -1130,16 +1130,16 @@
         <v>44</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="J4" s="9">
         <v>1</v>
@@ -1156,22 +1156,22 @@
         <v>2</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="E5" s="8" t="s">
         <v>45</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="J5" s="7">
         <v>12</v>
@@ -1194,16 +1194,16 @@
         <v>46</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J6" s="9">
         <v>1</v>
@@ -1226,16 +1226,16 @@
         <v>47</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="J7" s="7">
         <v>3</v>
@@ -1258,16 +1258,16 @@
         <v>48</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="J8" s="9">
         <v>3</v>
@@ -1290,16 +1290,16 @@
         <v>49</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
@@ -1316,22 +1316,22 @@
         <v>2</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>50</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="J10" s="9">
         <v>2</v>
@@ -1354,16 +1354,16 @@
         <v>51</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="J11" s="7">
         <v>2</v>
@@ -1386,23 +1386,23 @@
         <v>52</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
       </c>
       <c r="K12" s="9"/>
     </row>
-    <row r="13" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="11">
         <f>ROW(B13) - ROW($B$2)</f>
@@ -1414,20 +1414,20 @@
       <c r="D13" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="E13" s="8" t="s">
-        <v>53</v>
+      <c r="E13" s="10" t="s">
+        <v>168</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="G13" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>125</v>
+        <v>167</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>166</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="J13" s="7">
         <v>2</v>
@@ -1447,19 +1447,19 @@
         <v>22</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
@@ -1479,19 +1479,19 @@
         <v>23</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
@@ -1505,25 +1505,25 @@
         <v>14</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>24</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="J16" s="7">
         <v>1</v>
@@ -1540,22 +1540,22 @@
         <v>6</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="F17" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="H17" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="G17" s="10" t="s">
-        <v>160</v>
-      </c>
-      <c r="H17" s="9" t="s">
-        <v>161</v>
-      </c>
       <c r="I17" s="10" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="J17" s="7">
         <v>1</v>
@@ -1575,19 +1575,19 @@
         <v>25</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="J18" s="9">
         <v>6</v>
@@ -1607,19 +1607,19 @@
         <v>26</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="J19" s="9">
         <v>2</v>
@@ -1639,19 +1639,19 @@
         <v>27</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="J20" s="7">
         <v>2</v>
@@ -1671,19 +1671,19 @@
         <v>28</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="H21" s="9" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="J21" s="9">
         <v>7</v>
@@ -1703,19 +1703,19 @@
         <v>29</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I22" s="8" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="J22" s="7">
         <v>1</v>
@@ -1735,19 +1735,19 @@
         <v>30</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G23" s="10" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="H23" s="9" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I23" s="10" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="J23" s="9">
         <v>4</v>
@@ -1767,19 +1767,19 @@
         <v>31</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I24" s="8" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="J24" s="7">
         <v>2</v>
@@ -1799,19 +1799,19 @@
         <v>32</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G25" s="10" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="H25" s="9" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I25" s="10" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="J25" s="9">
         <v>2</v>
@@ -1831,19 +1831,19 @@
         <v>33</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I26" s="8" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="J26" s="7">
         <v>2</v>
@@ -1863,19 +1863,19 @@
         <v>34</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="J27" s="7">
         <v>1</v>
@@ -1895,19 +1895,19 @@
         <v>35</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="J28" s="9">
         <v>2</v>
@@ -1927,19 +1927,19 @@
         <v>36</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
@@ -1959,19 +1959,19 @@
         <v>37</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="J30" s="9">
         <v>1</v>
@@ -1988,22 +1988,22 @@
         <v>8</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="G31" s="10" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="H31" s="9" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I31" s="10" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="J31" s="9">
         <v>1</v>
@@ -2023,19 +2023,19 @@
         <v>38</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="G32" s="8" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="H32" s="7" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="I32" s="8" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="J32" s="7">
         <v>1</v>
@@ -2055,19 +2055,19 @@
         <v>39</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="G33" s="10" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="H33" s="9" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="J33" s="9">
         <v>1</v>
@@ -2087,19 +2087,19 @@
         <v>40</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="G34" s="8" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H34" s="7" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="I34" s="8" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="J34" s="7">
         <v>3</v>
@@ -2116,22 +2116,22 @@
         <v>10</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G35" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="H35" s="9" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="J35" s="9">
         <v>1</v>
@@ -2151,19 +2151,19 @@
         <v>41</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="G36" s="8" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="H36" s="7" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="I36" s="8" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="J36" s="7">
         <v>1</v>
@@ -2176,8 +2176,9 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="H18" r:id="rId1" display="https://www.lcsc.com/brand-detail/86.html"/>
+    <hyperlink ref="H13" r:id="rId2" display="https://www.lcsc.com/brand-detail/11578.html"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>